<commit_message>
Republish EU IG with updated dependencies
- Rebuild with corrected hl7.fhir.eu.extensions.r5 and hl7.terminology.r5 dependencies
- Update all generated files with dependency fixes

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/eu/0.0.1/StructureDefinition-Composition-eu-lab.xlsx
+++ b/docs/eu/0.0.1/StructureDefinition-Composition-eu-lab.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-15T17:07:07+02:00</t>
+    <t>2026-03-15T18:07:36+02:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -480,7 +480,7 @@
     <t>information-recipient</t>
   </si>
   <si>
-    <t xml:space="preserve">Extension {http://hl7.eu/fhir/StructureDefinition/information-recipient|0.1.1}
+    <t xml:space="preserve">Extension {http://hl7.eu/fhir/StructureDefinition/information-recipient|1.2.0}
 </t>
   </si>
   <si>

</xml_diff>